<commit_message>
major revisions to AlloyModel to support namespaces and overloading
</commit_message>
<xml_diff>
--- a/app/src/main/java/ca/uwaterloo/watform/alloymodel/scopeCalculations.xlsx
+++ b/app/src/main/java/ca/uwaterloo/watform/alloymodel/scopeCalculations.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nday/UW/github/dashplus/dashplus/app/src/main/java/ca/uwaterloo/watform/alloymodel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E20FA4B-CF19-B042-8D32-9EDE21D58010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0468C0B-C79D-FE4D-81D3-0BE1397BFD15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="18460" xr2:uid="{250CF1D8-1848-1049-9629-7130975B20CE}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="43460" windowHeight="25700" xr2:uid="{250CF1D8-1848-1049-9629-7130975B20CE}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="215" uniqueCount="44">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="53">
   <si>
     <t>nothing</t>
   </si>
@@ -254,9 +254,6 @@
   </si>
   <si>
     <t>There are 36 combinations below</t>
-  </si>
-  <si>
-    <t>Scope Set</t>
   </si>
   <si>
     <r>
@@ -303,6 +300,36 @@
   </si>
   <si>
     <t>error c !=m; override g &lt;= c</t>
+  </si>
+  <si>
+    <t>ScopeCmdProfile</t>
+  </si>
+  <si>
+    <t>multiple scopes for same sig?</t>
+  </si>
+  <si>
+    <t>non-zero value from child and nothing given for top-level parent is an error</t>
+  </si>
+  <si>
+    <t>abstact sigs don't seem to affect this</t>
+  </si>
+  <si>
+    <t>Alloy discourse</t>
+  </si>
+  <si>
+    <t>can set a scope for one sigs in command</t>
+  </si>
+  <si>
+    <t>cannot set a scope for enums parent in a command</t>
+  </si>
+  <si>
+    <t>top-level parent not set with no default -&gt; error</t>
+  </si>
+  <si>
+    <t>enum parent is always top-level</t>
+  </si>
+  <si>
+    <t>scope not given for a subsig then it takes parents scope</t>
   </si>
 </sst>
 </file>
@@ -386,7 +413,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -402,7 +429,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -757,7 +783,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DE9F18B8-9DE0-E84D-8F57-BBDF96F5BAC5}">
-  <dimension ref="A1:G60"/>
+  <dimension ref="A1:I60"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9" customWidth="1"/>
@@ -801,7 +827,7 @@
     </row>
     <row r="8" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A8" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:1" x14ac:dyDescent="0.2">
@@ -822,6 +848,11 @@
         <v>29</v>
       </c>
     </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13" t="s">
+        <v>46</v>
+      </c>
+    </row>
     <row r="14" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>30</v>
@@ -832,7 +863,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="18" spans="1:7" s="4" customFormat="1" ht="35" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:9" s="4" customFormat="1" ht="35" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
         <v>17</v>
       </c>
@@ -849,16 +880,16 @@
         <v>18</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="G18" s="4" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="17" thickTop="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:9" ht="17" thickTop="1" x14ac:dyDescent="0.2">
       <c r="E19" s="5"/>
     </row>
-    <row r="20" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>0</v>
       </c>
@@ -876,7 +907,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>0</v>
       </c>
@@ -893,7 +924,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>0</v>
       </c>
@@ -911,7 +942,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="23" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>0</v>
       </c>
@@ -931,7 +962,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="24" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>0</v>
       </c>
@@ -949,7 +980,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="25" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>0</v>
       </c>
@@ -969,11 +1000,11 @@
         <v>8</v>
       </c>
     </row>
-    <row r="26" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A26" s="1"/>
       <c r="E26" s="5"/>
     </row>
-    <row r="27" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>0</v>
       </c>
@@ -991,7 +1022,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="28" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>0</v>
       </c>
@@ -1011,7 +1042,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="29" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
         <v>0</v>
       </c>
@@ -1031,8 +1062,11 @@
       <c r="G29" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="30" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I29" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
         <v>0</v>
       </c>
@@ -1054,8 +1088,11 @@
       <c r="G30" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="31" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I30" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
         <v>0</v>
       </c>
@@ -1072,8 +1109,11 @@
       <c r="F31" t="s">
         <v>10</v>
       </c>
-    </row>
-    <row r="32" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I31" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A32" s="1">
         <v>0</v>
       </c>
@@ -1093,11 +1133,11 @@
         <v>10</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A33" s="1"/>
       <c r="E33" s="5"/>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A34" s="1">
         <v>0</v>
       </c>
@@ -1115,7 +1155,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
         <v>0</v>
       </c>
@@ -1134,8 +1174,11 @@
       <c r="F35" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I35" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A36" s="1">
         <v>0</v>
       </c>
@@ -1155,8 +1198,11 @@
       <c r="G36" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I36" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
         <v>0</v>
       </c>
@@ -1178,8 +1224,11 @@
       <c r="G37" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I37" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A38" s="1">
         <v>0</v>
       </c>
@@ -1200,7 +1249,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A39" s="1">
         <v>0</v>
       </c>
@@ -1222,11 +1271,14 @@
       <c r="G39" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I39" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" x14ac:dyDescent="0.2">
       <c r="E40" s="5"/>
     </row>
-    <row r="41" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>21</v>
       </c>
@@ -1243,8 +1295,11 @@
       <c r="F41" t="s">
         <v>24</v>
       </c>
-    </row>
-    <row r="42" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="I41" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>21</v>
       </c>
@@ -1261,7 +1316,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="43" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>21</v>
       </c>
@@ -1282,7 +1337,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>21</v>
       </c>
@@ -1305,7 +1360,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>21</v>
       </c>
@@ -1320,10 +1375,10 @@
       </c>
       <c r="E45" s="6"/>
       <c r="G45" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.2">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>21</v>
       </c>
@@ -1340,13 +1395,13 @@
         <v>21</v>
       </c>
       <c r="G46" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.2">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
       <c r="E47" s="5"/>
     </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>21</v>
       </c>
@@ -1404,7 +1459,7 @@
         <v>4</v>
       </c>
       <c r="E50" s="6"/>
-      <c r="F50" s="9" t="s">
+      <c r="F50" t="s">
         <v>15</v>
       </c>
       <c r="G50" t="s">
@@ -1427,7 +1482,7 @@
       <c r="E51" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="F51" s="9" t="s">
+      <c r="F51" t="s">
         <v>15</v>
       </c>
       <c r="G51" t="s">
@@ -1566,7 +1621,7 @@
         <v>6</v>
       </c>
       <c r="G58" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.2">

</xml_diff>